<commit_message>
feat(F-NAR-016): TREE-DIF-019 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-019.xlsx
+++ b/stories/arbres/TREE-DIF-019.xlsx
@@ -6423,12 +6423,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. Le vert de la feuille sent encore. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Sous les pieds, le sable chuchote encore. Un trou rond reste au milieu du bac.</t>
+          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. La pêche sent encore le soleil. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Sous les pieds, le sable chuchote encore. Un trou rond reste au milieu du bac.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. Le vert de la feuille sent encore. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Sous les pieds, le sable chuchote encore. Un trou rond reste au milieu du bac.</t>
+          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. La pêche sent encore le soleil. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Sous les pieds, le sable chuchote encore. Un trou rond reste au milieu du bac.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6567,7 +6567,7 @@
 enfant-f|Tu l'avais attaché, pile.
 copain|Il n'est pas parti.
 papa|Vous avez demandé, et ça a tenu.
-maman|Le vert de la feuille sent encore.
+maman|La pêche sent encore le soleil.
 narrateur|Trois bouches, un même sucré.
 narrateur|Le doudou reprend le sac, tout doux.
 narrateur|Sous les pieds, le sable chuchote encore.
@@ -11435,12 +11435,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. Le vert de la feuille sent encore. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Un petit toc dort encore dans le métal. Vide et chaud, le toboggan se tait.</t>
+          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. La pêche sent encore le soleil. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Un petit toc dort encore dans le métal. Vide et chaud, le toboggan se tait.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. Le vert de la feuille sent encore. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Un petit toc dort encore dans le métal. Vide et chaud, le toboggan se tait.</t>
+          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. La pêche sent encore le soleil. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Un petit toc dort encore dans le métal. Vide et chaud, le toboggan se tait.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11579,7 +11579,7 @@
 enfant-f|Tu l'avais attaché, pile.
 copain|Il n'est pas parti.
 papa|Vous avez demandé, et ça a tenu.
-maman|Le vert de la feuille sent encore.
+maman|La pêche sent encore le soleil.
 narrateur|Trois bouches, un même sucré.
 narrateur|Le doudou reprend le sac, tout doux.
 narrateur|Un petit toc dort encore dans le métal.
@@ -16447,12 +16447,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. Le vert de la feuille sent encore. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Puis la chaîne se tait, tout doux. Plus aucun cri sur la chaîne.</t>
+          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. La pêche sent encore le soleil. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Puis la chaîne se tait, tout doux. Plus aucun cri sur la chaîne.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. Le vert de la feuille sent encore. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Puis la chaîne se tait, tout doux. Plus aucun cri sur la chaîne.</t>
+          <t>Maman détache le doudou, plus tard. Tu l'avais attaché, pile. Il n'est pas parti. Vous avez demandé, et ça a tenu. La pêche sent encore le soleil. Trois bouches, un même sucré. Le doudou reprend le sac, tout doux. Puis la chaîne se tait, tout doux. Plus aucun cri sur la chaîne.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16591,7 +16591,7 @@
 enfant-f|Tu l'avais attaché, pile.
 copain|Il n'est pas parti.
 papa|Vous avez demandé, et ça a tenu.
-maman|Le vert de la feuille sent encore.
+maman|La pêche sent encore le soleil.
 narrateur|Trois bouches, un même sucré.
 narrateur|Le doudou reprend le sac, tout doux.
 narrateur|Puis la chaîne se tait, tout doux.
@@ -16616,7 +16616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16715,6 +16715,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>